<commit_message>
fix(excel): finalize 'Perfect Format' with fixed widths, HEX colors, and grid borders
</commit_message>
<xml_diff>
--- a/docs/samples/written/【ライフホープ寝屋川2番館様】訪問施術サービス申込書.xlsx
+++ b/docs/samples/written/【ライフホープ寝屋川2番館様】訪問施術サービス申込書.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd35f0bba0eb985b/デスクトップ/VEXUM/プラージュ様/-OCR-main/-OCR-main/docs/samples/written/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{CA7C3648-184A-4B53-8745-29CAD33D6874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69AF5219-5821-4784-BCBC-E58F642A1F78}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{CA7C3648-184A-4B53-8745-29CAD33D6874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABA4F0CE-10BB-4EB9-BE8E-FD554160975E}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8545FFEA-CFB0-4F4D-92CA-7457519C6A3D}"/>
   </bookViews>
@@ -43,9 +43,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="46">
   <si>
-    <t>【訪問理美容サービス　申込書】</t>
-  </si>
-  <si>
     <t>確認
 サイン欄</t>
     <rPh sb="0" eb="2">
@@ -346,6 +343,10 @@
   </si>
   <si>
     <t>※顔そり、シャンプーのみのご注文を承っておりません。</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>【訪問理美容サービス　申込書】</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -1816,7 +1817,7 @@
     <row r="1" spans="1:22" ht="31.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="1"/>
@@ -1836,7 +1837,7 @@
       <c r="R1" s="4"/>
       <c r="S1" s="4"/>
       <c r="T1" s="75" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U1" s="76"/>
       <c r="V1" s="1"/>
@@ -1866,7 +1867,7 @@
     <row r="3" spans="1:22" ht="19.5" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
       <c r="B3" s="7" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -1876,33 +1877,33 @@
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
       <c r="K3" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="L3" s="8" t="s">
         <v>3</v>
-      </c>
-      <c r="L3" s="8" t="s">
-        <v>4</v>
       </c>
       <c r="M3" s="8"/>
       <c r="N3" s="8"/>
       <c r="P3" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q3" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="R3" s="67"/>
       <c r="S3" s="4"/>
       <c r="T3" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="U3" s="10" t="s">
         <v>6</v>
-      </c>
-      <c r="U3" s="10" t="s">
-        <v>7</v>
       </c>
       <c r="V3" s="7"/>
     </row>
     <row r="4" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A4" s="6"/>
       <c r="B4" s="7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -1921,17 +1922,17 @@
       <c r="R4" s="68"/>
       <c r="S4" s="6"/>
       <c r="T4" s="11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U4" s="12" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="V4" s="6"/>
     </row>
     <row r="5" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A5" s="6"/>
       <c r="B5" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
@@ -1956,7 +1957,7 @@
     <row r="6" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A6" s="6"/>
       <c r="B6" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -1981,7 +1982,7 @@
     <row r="7" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A7" s="6"/>
       <c r="B7" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -2006,7 +2007,7 @@
     <row r="8" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A8" s="6"/>
       <c r="B8" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
@@ -2031,11 +2032,11 @@
     <row r="9" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A9" s="6"/>
       <c r="B9" s="99" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C9" s="99"/>
       <c r="D9" s="56" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
@@ -2093,17 +2094,17 @@
     <row r="12" spans="1:22" ht="16.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="13"/>
       <c r="B12" s="81" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="83" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="83" t="s">
+      <c r="D12" s="85" t="s">
         <v>16</v>
-      </c>
-      <c r="D12" s="85" t="s">
-        <v>17</v>
       </c>
       <c r="E12" s="86"/>
       <c r="F12" s="81" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G12" s="85"/>
       <c r="H12" s="85"/>
@@ -2113,26 +2114,26 @@
       <c r="L12" s="85"/>
       <c r="M12" s="100"/>
       <c r="N12" s="89" t="s">
+        <v>18</v>
+      </c>
+      <c r="O12" s="81" t="s">
         <v>19</v>
-      </c>
-      <c r="O12" s="81" t="s">
-        <v>20</v>
       </c>
       <c r="P12" s="91"/>
       <c r="Q12" s="92" t="s">
+        <v>20</v>
+      </c>
+      <c r="R12" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="R12" s="92" t="s">
+      <c r="S12" s="92" t="s">
         <v>22</v>
       </c>
-      <c r="S12" s="92" t="s">
+      <c r="T12" s="93" t="s">
         <v>23</v>
       </c>
-      <c r="T12" s="93" t="s">
+      <c r="U12" s="96" t="s">
         <v>24</v>
-      </c>
-      <c r="U12" s="96" t="s">
-        <v>25</v>
       </c>
       <c r="V12" s="97"/>
     </row>
@@ -2143,32 +2144,32 @@
       <c r="D13" s="87"/>
       <c r="E13" s="88"/>
       <c r="F13" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="G13" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="G13" s="15" t="s">
+      <c r="H13" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="H13" s="15" t="s">
+      <c r="I13" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="I13" s="16" t="s">
+      <c r="J13" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="J13" s="15" t="s">
+      <c r="K13" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="K13" s="15" t="s">
+      <c r="L13" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="L13" s="16" t="s">
+      <c r="M13" s="16" t="s">
         <v>32</v>
-      </c>
-      <c r="M13" s="16" t="s">
-        <v>33</v>
       </c>
       <c r="N13" s="90"/>
       <c r="O13" s="94" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="P13" s="95"/>
       <c r="Q13" s="84"/>
@@ -2210,10 +2211,10 @@
       </c>
       <c r="N14" s="90"/>
       <c r="O14" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="P14" s="20" t="s">
         <v>35</v>
-      </c>
-      <c r="P14" s="20" t="s">
-        <v>36</v>
       </c>
       <c r="Q14" s="84"/>
       <c r="R14" s="84"/>
@@ -2225,7 +2226,7 @@
     <row r="15" spans="1:22" s="25" customFormat="1" ht="16" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>
       <c r="B15" s="101" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C15" s="102"/>
       <c r="D15" s="103">
@@ -2281,17 +2282,17 @@
     <row r="16" spans="1:22" ht="16" x14ac:dyDescent="0.35">
       <c r="A16" s="26"/>
       <c r="B16" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="C16" s="27" t="s">
+      <c r="D16" s="105" t="s">
         <v>39</v>
-      </c>
-      <c r="D16" s="105" t="s">
-        <v>40</v>
       </c>
       <c r="E16" s="106"/>
       <c r="F16" s="28" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G16" s="61"/>
       <c r="H16" s="61"/>
@@ -2299,10 +2300,10 @@
       <c r="J16" s="29"/>
       <c r="K16" s="29"/>
       <c r="L16" s="29" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="M16" s="29" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N16" s="30">
         <v>4500</v>
@@ -2314,10 +2315,10 @@
         <v>0.60416666666666663</v>
       </c>
       <c r="Q16" s="31" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R16" s="31" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S16" s="32"/>
       <c r="T16" s="32"/>
@@ -2349,10 +2350,10 @@
       <c r="Q17" s="35"/>
       <c r="R17" s="52"/>
       <c r="S17" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T17" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U17" s="107"/>
       <c r="V17" s="107"/>
@@ -2382,10 +2383,10 @@
       <c r="Q18" s="39"/>
       <c r="R18" s="39"/>
       <c r="S18" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T18" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U18" s="108"/>
       <c r="V18" s="108"/>
@@ -2415,10 +2416,10 @@
       <c r="Q19" s="35"/>
       <c r="R19" s="35"/>
       <c r="S19" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T19" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U19" s="107"/>
       <c r="V19" s="107"/>
@@ -2448,10 +2449,10 @@
       <c r="Q20" s="53"/>
       <c r="R20" s="53"/>
       <c r="S20" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T20" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U20" s="108"/>
       <c r="V20" s="108"/>
@@ -2481,10 +2482,10 @@
       <c r="Q21" s="35"/>
       <c r="R21" s="35"/>
       <c r="S21" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T21" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U21" s="107"/>
       <c r="V21" s="107"/>
@@ -2514,10 +2515,10 @@
       <c r="Q22" s="53"/>
       <c r="R22" s="53"/>
       <c r="S22" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T22" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U22" s="108"/>
       <c r="V22" s="108"/>
@@ -2547,10 +2548,10 @@
       <c r="Q23" s="35"/>
       <c r="R23" s="35"/>
       <c r="S23" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T23" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U23" s="107"/>
       <c r="V23" s="107"/>
@@ -2580,10 +2581,10 @@
       <c r="Q24" s="53"/>
       <c r="R24" s="53"/>
       <c r="S24" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T24" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U24" s="108"/>
       <c r="V24" s="108"/>
@@ -2613,10 +2614,10 @@
       <c r="Q25" s="35"/>
       <c r="R25" s="35"/>
       <c r="S25" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T25" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U25" s="107"/>
       <c r="V25" s="107"/>
@@ -2646,10 +2647,10 @@
       <c r="Q26" s="53"/>
       <c r="R26" s="53"/>
       <c r="S26" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T26" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U26" s="108"/>
       <c r="V26" s="108"/>
@@ -2679,10 +2680,10 @@
       <c r="Q27" s="35"/>
       <c r="R27" s="35"/>
       <c r="S27" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T27" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U27" s="107"/>
       <c r="V27" s="107"/>
@@ -2712,10 +2713,10 @@
       <c r="Q28" s="53"/>
       <c r="R28" s="53"/>
       <c r="S28" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T28" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U28" s="108"/>
       <c r="V28" s="108"/>
@@ -2745,10 +2746,10 @@
       <c r="Q29" s="35"/>
       <c r="R29" s="35"/>
       <c r="S29" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T29" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U29" s="107"/>
       <c r="V29" s="107"/>
@@ -2778,10 +2779,10 @@
       <c r="Q30" s="53"/>
       <c r="R30" s="53"/>
       <c r="S30" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T30" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U30" s="108"/>
       <c r="V30" s="108"/>
@@ -2811,10 +2812,10 @@
       <c r="Q31" s="35"/>
       <c r="R31" s="35"/>
       <c r="S31" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T31" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U31" s="107"/>
       <c r="V31" s="107"/>
@@ -2843,10 +2844,10 @@
       <c r="Q32" s="53"/>
       <c r="R32" s="53"/>
       <c r="S32" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T32" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U32" s="108"/>
       <c r="V32" s="108"/>
@@ -2875,10 +2876,10 @@
       <c r="Q33" s="35"/>
       <c r="R33" s="35"/>
       <c r="S33" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T33" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U33" s="107"/>
       <c r="V33" s="107"/>
@@ -2907,10 +2908,10 @@
       <c r="Q34" s="53"/>
       <c r="R34" s="53"/>
       <c r="S34" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T34" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U34" s="108"/>
       <c r="V34" s="108"/>
@@ -2939,10 +2940,10 @@
       <c r="Q35" s="35"/>
       <c r="R35" s="35"/>
       <c r="S35" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T35" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U35" s="107"/>
       <c r="V35" s="107"/>
@@ -2971,10 +2972,10 @@
       <c r="Q36" s="53"/>
       <c r="R36" s="53"/>
       <c r="S36" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T36" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U36" s="108"/>
       <c r="V36" s="108"/>
@@ -3003,10 +3004,10 @@
       <c r="Q37" s="35"/>
       <c r="R37" s="35"/>
       <c r="S37" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T37" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U37" s="107"/>
       <c r="V37" s="107"/>
@@ -3035,10 +3036,10 @@
       <c r="Q38" s="53"/>
       <c r="R38" s="53"/>
       <c r="S38" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T38" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U38" s="108"/>
       <c r="V38" s="108"/>
@@ -3067,10 +3068,10 @@
       <c r="Q39" s="35"/>
       <c r="R39" s="35"/>
       <c r="S39" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T39" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U39" s="107"/>
       <c r="V39" s="107"/>
@@ -3099,10 +3100,10 @@
       <c r="Q40" s="53"/>
       <c r="R40" s="53"/>
       <c r="S40" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T40" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U40" s="108"/>
       <c r="V40" s="108"/>
@@ -3131,10 +3132,10 @@
       <c r="Q41" s="35"/>
       <c r="R41" s="35"/>
       <c r="S41" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T41" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U41" s="107"/>
       <c r="V41" s="107"/>
@@ -3163,10 +3164,10 @@
       <c r="Q42" s="53"/>
       <c r="R42" s="53"/>
       <c r="S42" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T42" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U42" s="108"/>
       <c r="V42" s="108"/>
@@ -3195,10 +3196,10 @@
       <c r="Q43" s="35"/>
       <c r="R43" s="35"/>
       <c r="S43" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T43" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U43" s="107"/>
       <c r="V43" s="107"/>
@@ -3227,10 +3228,10 @@
       <c r="Q44" s="53"/>
       <c r="R44" s="53"/>
       <c r="S44" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T44" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U44" s="108"/>
       <c r="V44" s="108"/>
@@ -3259,10 +3260,10 @@
       <c r="Q45" s="35"/>
       <c r="R45" s="35"/>
       <c r="S45" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T45" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U45" s="107"/>
       <c r="V45" s="107"/>
@@ -3291,10 +3292,10 @@
       <c r="Q46" s="53"/>
       <c r="R46" s="53"/>
       <c r="S46" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T46" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U46" s="108"/>
       <c r="V46" s="108"/>
@@ -3323,10 +3324,10 @@
       <c r="Q47" s="35"/>
       <c r="R47" s="35"/>
       <c r="S47" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T47" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U47" s="107"/>
       <c r="V47" s="107"/>
@@ -3355,10 +3356,10 @@
       <c r="Q48" s="53"/>
       <c r="R48" s="53"/>
       <c r="S48" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T48" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U48" s="108"/>
       <c r="V48" s="108"/>
@@ -3387,10 +3388,10 @@
       <c r="Q49" s="35"/>
       <c r="R49" s="35"/>
       <c r="S49" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T49" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U49" s="107"/>
       <c r="V49" s="107"/>
@@ -3419,10 +3420,10 @@
       <c r="Q50" s="53"/>
       <c r="R50" s="53"/>
       <c r="S50" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T50" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U50" s="108"/>
       <c r="V50" s="108"/>
@@ -3451,10 +3452,10 @@
       <c r="Q51" s="35"/>
       <c r="R51" s="35"/>
       <c r="S51" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T51" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U51" s="107"/>
       <c r="V51" s="107"/>
@@ -3483,10 +3484,10 @@
       <c r="Q52" s="53"/>
       <c r="R52" s="53"/>
       <c r="S52" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T52" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U52" s="108"/>
       <c r="V52" s="108"/>
@@ -3515,10 +3516,10 @@
       <c r="Q53" s="35"/>
       <c r="R53" s="35"/>
       <c r="S53" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T53" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U53" s="107"/>
       <c r="V53" s="107"/>
@@ -3547,10 +3548,10 @@
       <c r="Q54" s="53"/>
       <c r="R54" s="53"/>
       <c r="S54" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T54" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U54" s="108"/>
       <c r="V54" s="108"/>
@@ -3579,10 +3580,10 @@
       <c r="Q55" s="35"/>
       <c r="R55" s="35"/>
       <c r="S55" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T55" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U55" s="107"/>
       <c r="V55" s="107"/>
@@ -3611,10 +3612,10 @@
       <c r="Q56" s="53"/>
       <c r="R56" s="53"/>
       <c r="S56" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T56" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U56" s="108"/>
       <c r="V56" s="108"/>
@@ -3643,10 +3644,10 @@
       <c r="Q57" s="35"/>
       <c r="R57" s="35"/>
       <c r="S57" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T57" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U57" s="107"/>
       <c r="V57" s="107"/>
@@ -3675,10 +3676,10 @@
       <c r="Q58" s="53"/>
       <c r="R58" s="53"/>
       <c r="S58" s="40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T58" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U58" s="108"/>
       <c r="V58" s="108"/>
@@ -3707,10 +3708,10 @@
       <c r="Q59" s="35"/>
       <c r="R59" s="35"/>
       <c r="S59" s="36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T59" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="U59" s="107"/>
       <c r="V59" s="107"/>

</xml_diff>